<commit_message>
change BOM for D5,D6 due to JLC production issue
</commit_message>
<xml_diff>
--- a/Project Outputs for UZ_A_MAX11331/Rev02/BOM/BOM_JLC-UZ_A_MAX11331(Differential_Input)_13Dez2024.xlsx
+++ b/Project Outputs for UZ_A_MAX11331/Rev02/BOM/BOM_JLC-UZ_A_MAX11331(Differential_Input)_13Dez2024.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20416"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ga92wum\git\UltraZohm\PCB\uz_a_max11331\Project Outputs for UZ_A_MAX11331\Rev02\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:40009_{E35A7B6E-8D21-48FD-8349-E85315B3CE1E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BE41EB5-B41D-4F8B-9997-36C11ABDD6C2}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="24620" windowHeight="11120"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="24620" windowHeight="11120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="2" r:id="rId1"/>
@@ -23,15 +23,15 @@
 </file>
 
 <file path=xl/connections.xml><?xml version="1.0" encoding="utf-8"?>
-<connections xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <connection id="1" keepAlive="1" name="Abfrage - BOM_JLC-UZ_A_MAX11331(Differential_Input)" description="Verbindung mit der Abfrage 'BOM_JLC-UZ_A_MAX11331(Differential_Input)' in der Arbeitsmappe." type="5" refreshedVersion="6" background="1" saveData="1">
+<connections xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16">
+  <connection id="1" xr16:uid="{00000000-0015-0000-FFFF-FFFF00000000}" keepAlive="1" name="Abfrage - BOM_JLC-UZ_A_MAX11331(Differential_Input)" description="Verbindung mit der Abfrage 'BOM_JLC-UZ_A_MAX11331(Differential_Input)' in der Arbeitsmappe." type="5" refreshedVersion="6" background="1" saveData="1">
     <dbPr connection="Provider=Microsoft.Mashup.OleDb.1;Data Source=$Workbook$;Location=BOM_JLC-UZ_A_MAX11331(Differential_Input);Extended Properties=&quot;&quot;" command="SELECT * FROM [BOM_JLC-UZ_A_MAX11331(Differential_Input)]"/>
   </connection>
 </connections>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="593" uniqueCount="319">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="595" uniqueCount="321">
   <si>
     <t>Quantity</t>
   </si>
@@ -988,12 +988,18 @@
   </si>
   <si>
     <t>C16430</t>
+  </si>
+  <si>
+    <t>C15874 </t>
+  </si>
+  <si>
+    <t>Am 16.12.24 via Chat geändert, da C263143 nicht verfügbar bzw. auffindbar war.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1535,7 +1541,7 @@
 </file>
 
 <file path=xl/queryTables/queryTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="ExterneDaten_1" connectionId="1" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0">
+<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="ExterneDaten_1" connectionId="1" xr16:uid="{00000000-0016-0000-0000-000000000000}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0">
   <queryTableRefresh nextId="13" unboundColumnsRight="1">
     <queryTableFields count="12">
       <queryTableField id="1" name="Quantity" tableColumnId="1"/>
@@ -1556,24 +1562,24 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BOM_JLC_UZ_A_MAX11331_Differential_Input" displayName="BOM_JLC_UZ_A_MAX11331_Differential_Input" ref="A1:L59" tableType="queryTable" totalsRowShown="0">
-  <autoFilter ref="A1:L59"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="BOM_JLC_UZ_A_MAX11331_Differential_Input" displayName="BOM_JLC_UZ_A_MAX11331_Differential_Input" ref="A1:L59" tableType="queryTable" totalsRowShown="0">
+  <autoFilter ref="A1:L59" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <sortState ref="A2:K59">
     <sortCondition ref="C1"/>
   </sortState>
   <tableColumns count="12">
-    <tableColumn id="1" uniqueName="1" name="Quantity" queryTableFieldId="1"/>
-    <tableColumn id="2" uniqueName="2" name="Comment" queryTableFieldId="2"/>
-    <tableColumn id="3" uniqueName="3" name="Designator" queryTableFieldId="3"/>
-    <tableColumn id="4" uniqueName="4" name="Manufacturer" queryTableFieldId="4"/>
-    <tableColumn id="5" uniqueName="5" name="Value" queryTableFieldId="5"/>
-    <tableColumn id="6" uniqueName="6" name="Description" queryTableFieldId="6"/>
-    <tableColumn id="7" uniqueName="7" name="Footprint" queryTableFieldId="7"/>
-    <tableColumn id="8" uniqueName="8" name="Voltage" queryTableFieldId="8"/>
-    <tableColumn id="9" uniqueName="9" name="Dielectric" queryTableFieldId="9"/>
-    <tableColumn id="10" uniqueName="10" name="Manufacturer Part Number" queryTableFieldId="10"/>
-    <tableColumn id="11" uniqueName="11" name="LCSC Part Number" queryTableFieldId="11"/>
-    <tableColumn id="12" uniqueName="12" name="LCSC Alternative" queryTableFieldId="12"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" uniqueName="1" name="Quantity" queryTableFieldId="1"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" uniqueName="2" name="Comment" queryTableFieldId="2"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" uniqueName="3" name="Designator" queryTableFieldId="3"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" uniqueName="4" name="Manufacturer" queryTableFieldId="4"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" uniqueName="5" name="Value" queryTableFieldId="5"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" uniqueName="6" name="Description" queryTableFieldId="6"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" uniqueName="7" name="Footprint" queryTableFieldId="7"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" uniqueName="8" name="Voltage" queryTableFieldId="8"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" uniqueName="9" name="Dielectric" queryTableFieldId="9"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" uniqueName="10" name="Manufacturer Part Number" queryTableFieldId="10"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" uniqueName="11" name="LCSC Part Number" queryTableFieldId="11"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" uniqueName="12" name="LCSC Alternative" queryTableFieldId="12"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1875,8 +1881,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L69"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:N69"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.453125" bestFit="1" customWidth="1"/>
@@ -2455,7 +2461,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>2</v>
       </c>
@@ -2490,7 +2496,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>48</v>
       </c>
@@ -2525,7 +2531,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>1</v>
       </c>
@@ -2560,7 +2566,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>1</v>
       </c>
@@ -2595,7 +2601,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>1</v>
       </c>
@@ -2630,7 +2636,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>24</v>
       </c>
@@ -2665,7 +2671,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>2</v>
       </c>
@@ -2697,10 +2703,16 @@
         <v>121</v>
       </c>
       <c r="K23" t="s">
+        <v>319</v>
+      </c>
+      <c r="L23" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="N23" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>11</v>
       </c>
@@ -2735,7 +2747,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>2</v>
       </c>
@@ -2770,7 +2782,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>1</v>
       </c>
@@ -2805,7 +2817,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>1</v>
       </c>
@@ -2840,7 +2852,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>48</v>
       </c>
@@ -2875,7 +2887,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>48</v>
       </c>
@@ -2910,7 +2922,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A30">
         <v>1</v>
       </c>
@@ -2945,7 +2957,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A31">
         <v>2</v>
       </c>
@@ -2980,7 +2992,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A32">
         <v>1</v>
       </c>
@@ -3992,8 +4004,9 @@
     <sortCondition ref="K74"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>